<commit_message>
Prior scan MCMC-ABC + ReadMe Q1
</commit_message>
<xml_diff>
--- a/MCMC-ABC_results/baseline_metrics.xlsx
+++ b/MCMC-ABC_results/baseline_metrics.xlsx
@@ -487,7 +487,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Baseline — ε=0.5  N_DATASETS=5  N_ITER=100000</t>
+          <t>Baseline — ε=0.6  N_DATASETS=1  N_ITER=50000</t>
         </is>
       </c>
     </row>
@@ -537,10 +537,12 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>-0.02942</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>0.00223</v>
+        <v>-0.04092</v>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
@@ -560,10 +562,12 @@
         </is>
       </c>
       <c r="C5" s="5" t="n">
-        <v>0.08305</v>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>0.00404</v>
+        <v>0.10713</v>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
@@ -583,10 +587,12 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>0.03384</v>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>0.00078</v>
+        <v>0.03805</v>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
@@ -606,10 +612,12 @@
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>0.0641</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>0.0008</v>
+        <v>0.06981999999999999</v>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
@@ -628,11 +636,11 @@
           <t>std des 8 médianes inter-chaînes</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
-        <v>0.0009</v>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>0.00017</v>
+      <c r="C8" s="4" t="n"/>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
@@ -651,11 +659,11 @@
           <t>std des 8 médianes inter-chaînes</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n">
-        <v>0.00183</v>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>0.00066</v>
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
@@ -675,10 +683,12 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>0.12434</v>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>0.00334</v>
+        <v>0.14067</v>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
@@ -698,10 +708,12 @@
         </is>
       </c>
       <c r="C11" s="5" t="n">
-        <v>0.2386</v>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>0.00206</v>
+        <v>0.26349</v>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
@@ -720,11 +732,11 @@
           <t>Gelman-Rubin (cible &lt; 1.01)</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n">
-        <v>1.00018</v>
-      </c>
-      <c r="D12" s="4" t="n">
-        <v>9.000000000000001e-05</v>
+      <c r="C12" s="4" t="n"/>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
@@ -743,11 +755,11 @@
           <t>Gelman-Rubin (cible &lt; 1.01)</t>
         </is>
       </c>
-      <c r="C13" s="5" t="n">
-        <v>1.00024</v>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>0.00013</v>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
@@ -767,10 +779,12 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>0.00349</v>
-      </c>
-      <c r="D14" s="4" t="n">
-        <v>0.00018</v>
+        <v>0.02145</v>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
@@ -790,10 +804,12 @@
         </is>
       </c>
       <c r="C15" s="5" t="n">
-        <v>0.00241</v>
-      </c>
-      <c r="D15" s="5" t="n">
-        <v>8.000000000000001e-05</v>
+        <v>0.01527</v>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
@@ -813,10 +829,12 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>0.05362</v>
-      </c>
-      <c r="D16" s="4" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.06347</v>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Last update before big run
</commit_message>
<xml_diff>
--- a/MCMC-ABC_results/baseline_metrics.xlsx
+++ b/MCMC-ABC_results/baseline_metrics.xlsx
@@ -487,7 +487,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Baseline — ε=0.6  N_DATASETS=1  N_ITER=50000</t>
+          <t>Baseline — ε=0.6  N_DATASETS=5  N_ITER=40000</t>
         </is>
       </c>
     </row>
@@ -537,12 +537,10 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>-0.04092</v>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>-0.03895</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>0.00256</v>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
@@ -562,12 +560,10 @@
         </is>
       </c>
       <c r="C5" s="5" t="n">
-        <v>0.10713</v>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>0.10354</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>0.00303</v>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
@@ -587,12 +583,10 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>0.03805</v>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>0.03962</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>0.00094</v>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
@@ -612,12 +606,10 @@
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>0.06981999999999999</v>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>0.00136</v>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
@@ -636,11 +628,11 @@
           <t>std des 8 médianes inter-chaînes</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="C8" s="4" t="n">
+        <v>0.00195</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>0.00099</v>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
@@ -659,11 +651,11 @@
           <t>std des 8 médianes inter-chaînes</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="C9" s="5" t="n">
+        <v>0.00359</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>0.00166</v>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
@@ -683,12 +675,10 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>0.14067</v>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>0.14437</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>0.00346</v>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
@@ -708,12 +698,10 @@
         </is>
       </c>
       <c r="C11" s="5" t="n">
-        <v>0.26349</v>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>0.25858</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>0.00455</v>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
@@ -732,11 +720,11 @@
           <t>Gelman-Rubin (cible &lt; 1.01)</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="C12" s="4" t="n">
+        <v>1.00077</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>0.00059</v>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
@@ -755,11 +743,11 @@
           <t>Gelman-Rubin (cible &lt; 1.01)</t>
         </is>
       </c>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="C13" s="5" t="n">
+        <v>1.00112</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>0.0006400000000000001</v>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
@@ -779,12 +767,10 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>0.02145</v>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>0.00409</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>0.00029</v>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
@@ -804,12 +790,10 @@
         </is>
       </c>
       <c r="C15" s="5" t="n">
-        <v>0.01527</v>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>0.00297</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>0.00032</v>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
@@ -829,12 +813,10 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>0.06347</v>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>0.06655</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>0.0015</v>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>

</xml_diff>